<commit_message>
Added some Updates in feature
</commit_message>
<xml_diff>
--- a/src/test/resources/register_data.xlsx
+++ b/src/test/resources/register_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SeleniumJavaAutomationProject\Automation-Project\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E21E659F-2F6E-4ACD-B77C-76C81F48C6EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D7FF9DE-72AA-4E47-B0E8-D0B215B75F26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3984" yWindow="1752" windowWidth="17280" windowHeight="9948" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,7 +54,7 @@
     <t>bad100</t>
   </si>
   <si>
-    <t>bad007@gmail.com</t>
+    <t>bad143@gmail.com</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Checked execution of failed test
</commit_message>
<xml_diff>
--- a/src/test/resources/register_data.xlsx
+++ b/src/test/resources/register_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SeleniumJavaAutomationProject\Automation-Project\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AD932B0-F53B-46F0-8F6C-18B2CDCD8A59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{324D4FBA-1DDD-4E18-A7FB-76C96524A489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3984" yWindow="1752" windowWidth="17280" windowHeight="9948" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,7 +54,7 @@
     <t>bad100</t>
   </si>
   <si>
-    <t>bad153@gmail.com</t>
+    <t>bad163@gmail.com</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Solved Add to Cart Locator
</commit_message>
<xml_diff>
--- a/src/test/resources/register_data.xlsx
+++ b/src/test/resources/register_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SeleniumJavaAutomationProject\Automation-Project\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3DE6C18-FAB2-49A7-89CD-10CEEC0BF520}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6303F42C-F862-42B7-8D76-43CCE5689F63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3984" yWindow="1752" windowWidth="17280" windowHeight="9948" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,7 +54,7 @@
     <t>bad100</t>
   </si>
   <si>
-    <t>bad134@gmail.com</t>
+    <t>bad102@gmail.com</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Added Requriments in folder
</commit_message>
<xml_diff>
--- a/src/test/resources/register_data.xlsx
+++ b/src/test/resources/register_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SeleniumJavaAutomationProject\Automation-Project\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30790127-2DD2-4978-9BBF-B29A7429E1EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69282C3D-1419-40D2-8D7F-2109DFF260C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,7 +54,7 @@
     <t>bad100</t>
   </si>
   <si>
-    <t>tilo009@gmail.com</t>
+    <t>tilo010@gmail.com</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Added logout feature and step definition
</commit_message>
<xml_diff>
--- a/src/test/resources/register_data.xlsx
+++ b/src/test/resources/register_data.xlsx
@@ -3,22 +3,21 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SeleniumJavaAutomationProject\Automation-Project\src\test\resources\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4082F33E-6F42-42F6-904F-D9BD909C039F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{D86394EF-466C-4038-AD24-B0F3A615140E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="registerVData" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="2"/>
     </ext>
   </extLst>
 </workbook>
@@ -54,7 +53,7 @@
     <t>bad100</t>
   </si>
   <si>
-    <t>tilo013@gmail.com</t>
+    <t>tilo0jb13@gmail.com</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Added new feature Account
</commit_message>
<xml_diff>
--- a/src/test/resources/register_data.xlsx
+++ b/src/test/resources/register_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SeleniumJavaAutomationProject\Automation-Project\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4082F33E-6F42-42F6-904F-D9BD909C039F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F68F000-A8AE-46B5-AAD1-5E1110D923A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,7 +54,7 @@
     <t>bad100</t>
   </si>
   <si>
-    <t>tilo013@gmail.com</t>
+    <t>tilo077@gmail.com</t>
   </si>
 </sst>
 </file>

</xml_diff>